<commit_message>
France daily ratings for 2026-03-17
</commit_message>
<xml_diff>
--- a/output/daily_ratings/france_ratings_2026-03-17.xlsx
+++ b/output/daily_ratings/france_ratings_2026-03-17.xlsx
@@ -576,10 +576,10 @@
         <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P2" t="n">
-        <v>122.2469253554297</v>
+        <v>120.5898501797769</v>
       </c>
       <c r="Q2" t="n">
         <v>-1.438970000000012</v>
@@ -588,10 +588,10 @@
         <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>92.58707204518741</v>
+        <v>91.27322201459462</v>
       </c>
       <c r="T2" t="n">
-        <v>92.58707204518741</v>
+        <v>91.27322201459462</v>
       </c>
     </row>
     <row r="3">
@@ -650,10 +650,10 @@
         <v>1.75</v>
       </c>
       <c r="O3" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P3" t="n">
-        <v>116.0987123226217</v>
+        <v>114.4603948074345</v>
       </c>
       <c r="Q3" t="n">
         <v>7.379509999999982</v>
@@ -662,10 +662,10 @@
         <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>94.48868352654371</v>
+        <v>93.04657208903488</v>
       </c>
       <c r="T3" t="n">
-        <v>94.48868352654371</v>
+        <v>93.04657208903488</v>
       </c>
     </row>
     <row r="4">
@@ -724,10 +724,10 @@
         <v>1.9</v>
       </c>
       <c r="O4" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P4" t="n">
-        <v>115.5717226340952</v>
+        <v>113.9350129183766</v>
       </c>
       <c r="Q4" t="n">
         <v>6.277199999999993</v>
@@ -736,10 +736,10 @@
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>93.32838943148165</v>
+        <v>91.97314661611868</v>
       </c>
       <c r="T4" t="n">
-        <v>93.32838943148165</v>
+        <v>91.97314661611868</v>
       </c>
     </row>
     <row r="5">
@@ -798,10 +798,10 @@
         <v>2.4</v>
       </c>
       <c r="O5" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P5" t="n">
-        <v>113.8150903390072</v>
+        <v>112.1837399548502</v>
       </c>
       <c r="Q5" t="n">
         <v>4.072579999999988</v>
@@ -810,10 +810,10 @@
         <v>0</v>
       </c>
       <c r="S5" t="n">
-        <v>90.50741200209379</v>
+        <v>89.36432592731073</v>
       </c>
       <c r="T5" t="n">
-        <v>90.50741200209379</v>
+        <v>89.36432592731073</v>
       </c>
     </row>
     <row r="6">
@@ -872,10 +872,10 @@
         <v>3.65</v>
       </c>
       <c r="O6" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P6" t="n">
-        <v>109.4235096012872</v>
+        <v>107.8055575460342</v>
       </c>
       <c r="Q6" t="n">
         <v>-3.643590000000017</v>
@@ -884,10 +884,10 @@
         <v>0</v>
       </c>
       <c r="S6" t="n">
-        <v>81.88496409739561</v>
+        <v>81.38837787392173</v>
       </c>
       <c r="T6" t="n">
-        <v>81.88496409739561</v>
+        <v>81.38837787392173</v>
       </c>
     </row>
     <row r="7">
@@ -946,10 +946,10 @@
         <v>4.4</v>
       </c>
       <c r="O7" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P7" t="n">
-        <v>106.7885611586551</v>
+        <v>105.1786481007446</v>
       </c>
       <c r="Q7" t="n">
         <v>5.174889999999976</v>
@@ -958,10 +958,10 @@
         <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>86.28852177507061</v>
+        <v>85.47157666323976</v>
       </c>
       <c r="T7" t="n">
-        <v>86.28852177507061</v>
+        <v>85.47157666323976</v>
       </c>
     </row>
     <row r="8">
@@ -1020,10 +1020,10 @@
         <v>4.9</v>
       </c>
       <c r="O8" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P8" t="n">
-        <v>105.0319288635671</v>
+        <v>103.4273751372182</v>
       </c>
       <c r="Q8" t="n">
         <v>1.867959999999982</v>
@@ -1032,10 +1032,10 @@
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>82.68254218006849</v>
+        <v>82.13580780874723</v>
       </c>
       <c r="T8" t="n">
-        <v>82.68254218006849</v>
+        <v>82.13580780874723</v>
       </c>
     </row>
     <row r="9">
@@ -1094,10 +1094,10 @@
         <v>5.9</v>
       </c>
       <c r="O9" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P9" t="n">
-        <v>101.518664273391</v>
+        <v>99.9248292101654</v>
       </c>
       <c r="Q9" t="n">
         <v>-6.950520000000012</v>
@@ -1106,10 +1106,10 @@
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>73.90057865883576</v>
+        <v>74.01037376839314</v>
       </c>
       <c r="T9" t="n">
-        <v>73.90057865883576</v>
+        <v>74.01037376839314</v>
       </c>
     </row>
     <row r="10">
@@ -1168,10 +1168,10 @@
         <v>6.15</v>
       </c>
       <c r="O10" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P10" t="n">
-        <v>100.640348125847</v>
+        <v>99.0491927284022</v>
       </c>
       <c r="Q10" t="n">
         <v>-2.541280000000015</v>
@@ -1180,10 +1180,10 @@
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>76.41510077221309</v>
+        <v>76.34070425241187</v>
       </c>
       <c r="T10" t="n">
-        <v>76.41510077221309</v>
+        <v>76.34070425241187</v>
       </c>
     </row>
     <row r="11">
@@ -1242,10 +1242,10 @@
         <v>6.300000000000001</v>
       </c>
       <c r="O11" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P11" t="n">
-        <v>100.1133584373206</v>
+        <v>98.52381083934428</v>
       </c>
       <c r="Q11" t="n">
         <v>-4.745900000000006</v>
@@ -1254,10 +1254,10 @@
         <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>74.46980451153678</v>
+        <v>74.54033061381112</v>
       </c>
       <c r="T11" t="n">
-        <v>74.46980451153678</v>
+        <v>74.54033061381112</v>
       </c>
     </row>
     <row r="12">
@@ -1316,10 +1316,10 @@
         <v>9.300000000000001</v>
       </c>
       <c r="O12" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P12" t="n">
-        <v>89.57356466679246</v>
+        <v>88.0161730581859</v>
       </c>
       <c r="Q12" t="n">
         <v>-1.438970000000012</v>
@@ -1328,10 +1328,10 @@
         <v>0</v>
       </c>
       <c r="S12" t="n">
-        <v>69.31897241942342</v>
+        <v>69.7916289662315</v>
       </c>
       <c r="T12" t="n">
-        <v>69.31897241942342</v>
+        <v>69.7916289662315</v>
       </c>
     </row>
     <row r="13">
@@ -1390,10 +1390,10 @@
         <v>9.550000000000001</v>
       </c>
       <c r="O13" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P13" t="n">
-        <v>88.69524851924845</v>
+        <v>87.1405365764227</v>
       </c>
       <c r="Q13" t="n">
         <v>2.970269999999999</v>
@@ -1402,10 +1402,10 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>71.83349453280076</v>
+        <v>72.12195945025023</v>
       </c>
       <c r="T13" t="n">
-        <v>71.83349453280076</v>
+        <v>72.12195945025023</v>
       </c>
     </row>
     <row r="14">
@@ -1464,10 +1464,10 @@
         <v>12.55</v>
       </c>
       <c r="O14" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P14" t="n">
-        <v>78.15545474872029</v>
+        <v>76.63289879526431</v>
       </c>
       <c r="Q14" t="n">
         <v>-2.541280000000015</v>
@@ -1476,10 +1476,10 @@
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>60.40264511577335</v>
+        <v>61.55767247719424</v>
       </c>
       <c r="T14" t="n">
-        <v>60.40264511577335</v>
+        <v>61.55767247719424</v>
       </c>
     </row>
     <row r="15">
@@ -1538,10 +1538,10 @@
         <v>13.8</v>
       </c>
       <c r="O15" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P15" t="n">
-        <v>73.76387401100023</v>
+        <v>72.25471638644831</v>
       </c>
       <c r="Q15" t="n">
         <v>-2.541280000000015</v>
@@ -1550,10 +1550,10 @@
         <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>57.27521237037496</v>
+        <v>58.67036158359704</v>
       </c>
       <c r="T15" t="n">
-        <v>57.27521237037496</v>
+        <v>58.67036158359704</v>
       </c>
     </row>
     <row r="16">
@@ -1612,10 +1612,10 @@
         <v>20.8</v>
       </c>
       <c r="O16" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P16" t="n">
-        <v>53.03491862529398</v>
+        <v>53.06855909137155</v>
       </c>
       <c r="Q16" t="n">
         <v>-3.643590000000017</v>
@@ -1684,10 +1684,10 @@
         <v>0</v>
       </c>
       <c r="O17" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P17" t="n">
-        <v>95.81399919387054</v>
+        <v>94.27182544794317</v>
       </c>
       <c r="Q17" t="n">
         <v>0.7656499999999937</v>
@@ -1696,10 +1696,10 @@
         <v>4.069673109043189</v>
       </c>
       <c r="S17" t="n">
-        <v>78.23124600528199</v>
+        <v>78.05484067299302</v>
       </c>
       <c r="T17" t="n">
-        <v>78.23124600528199</v>
+        <v>78.05484067299302</v>
       </c>
     </row>
     <row r="18">
@@ -1758,10 +1758,10 @@
         <v>0.15</v>
       </c>
       <c r="O18" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P18" t="n">
-        <v>95.29836931162072</v>
+        <v>93.75776870738601</v>
       </c>
       <c r="Q18" t="n">
         <v>4.072579999999988</v>
@@ -1770,10 +1770,10 @@
         <v>4.069673109043189</v>
       </c>
       <c r="S18" t="n">
-        <v>80.21905037729458</v>
+        <v>79.8966765385312</v>
       </c>
       <c r="T18" t="n">
-        <v>80.21905037729458</v>
+        <v>79.8966765385312</v>
       </c>
     </row>
     <row r="19">
@@ -1832,10 +1832,10 @@
         <v>0.2</v>
       </c>
       <c r="O19" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P19" t="n">
-        <v>95.12649268420411</v>
+        <v>93.58641646053361</v>
       </c>
       <c r="Q19" t="n">
         <v>-1.438970000000012</v>
@@ -1844,10 +1844,10 @@
         <v>4.069673109043189</v>
       </c>
       <c r="S19" t="n">
-        <v>76.17163884094658</v>
+        <v>76.14893283293665</v>
       </c>
       <c r="T19" t="n">
-        <v>76.17163884094658</v>
+        <v>76.14893283293665</v>
       </c>
     </row>
     <row r="20">
@@ -1906,10 +1906,10 @@
         <v>1.45</v>
       </c>
       <c r="O20" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P20" t="n">
-        <v>90.82957699878894</v>
+        <v>89.30261028922386</v>
       </c>
       <c r="Q20" t="n">
         <v>-2.541280000000015</v>
@@ -1918,10 +1918,10 @@
         <v>4.069673109043189</v>
       </c>
       <c r="S20" t="n">
-        <v>72.32661896841434</v>
+        <v>72.59691273795657</v>
       </c>
       <c r="T20" t="n">
-        <v>72.32661896841434</v>
+        <v>72.59691273795657</v>
       </c>
     </row>
     <row r="21">
@@ -1980,10 +1980,10 @@
         <v>2.7</v>
       </c>
       <c r="O21" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P21" t="n">
-        <v>86.53266131337375</v>
+        <v>85.0188041179141</v>
       </c>
       <c r="Q21" t="n">
         <v>4.072579999999988</v>
@@ -1992,10 +1992,10 @@
         <v>4.069673109043189</v>
       </c>
       <c r="S21" t="n">
-        <v>73.97661425518187</v>
+        <v>74.13352980276831</v>
       </c>
       <c r="T21" t="n">
-        <v>73.97661425518187</v>
+        <v>74.13352980276831</v>
       </c>
     </row>
     <row r="22">
@@ -2054,10 +2054,10 @@
         <v>2.85</v>
       </c>
       <c r="O22" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P22" t="n">
-        <v>86.01703143112394</v>
+        <v>84.50474737735694</v>
       </c>
       <c r="Q22" t="n">
         <v>-9.155140000000017</v>
@@ -2066,10 +2066,10 @@
         <v>4.069673109043189</v>
       </c>
       <c r="S22" t="n">
-        <v>64.18938614298067</v>
+        <v>65.07114318303832</v>
       </c>
       <c r="T22" t="n">
-        <v>64.18938614298067</v>
+        <v>65.07114318303832</v>
       </c>
     </row>
     <row r="23">
@@ -2128,10 +2128,10 @@
         <v>3.6</v>
       </c>
       <c r="O23" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P23" t="n">
-        <v>83.43888201987482</v>
+        <v>81.93446367457108</v>
       </c>
       <c r="Q23" t="n">
         <v>-9.155140000000017</v>
@@ -2140,10 +2140,10 @@
         <v>4.069673109043189</v>
       </c>
       <c r="S23" t="n">
-        <v>62.35337551882986</v>
+        <v>63.37610002546101</v>
       </c>
       <c r="T23" t="n">
-        <v>62.35337551882986</v>
+        <v>63.37610002546101</v>
       </c>
     </row>
     <row r="24">
@@ -2204,10 +2204,10 @@
         <v>0</v>
       </c>
       <c r="O24" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P24" t="n">
-        <v>108.8589025357003</v>
+        <v>102.2747076641523</v>
       </c>
       <c r="Q24" t="n">
         <v>1.867959999999982</v>
@@ -2216,10 +2216,10 @@
         <v>0</v>
       </c>
       <c r="S24" t="n">
-        <v>85.40789405057073</v>
+        <v>81.37565004442551</v>
       </c>
       <c r="T24" t="n">
-        <v>85.40789405057073</v>
+        <v>81.37565004442551</v>
       </c>
     </row>
     <row r="25">
@@ -2278,10 +2278,10 @@
         <v>1.5</v>
       </c>
       <c r="O25" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P25" t="n">
-        <v>104.7164571205546</v>
+        <v>98.13138057520885</v>
       </c>
       <c r="Q25" t="n">
         <v>1.867959999999982</v>
@@ -2290,10 +2290,10 @@
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>82.45788123944845</v>
+        <v>78.64322084833863</v>
       </c>
       <c r="T25" t="n">
-        <v>82.45788123944845</v>
+        <v>78.64322084833863</v>
       </c>
     </row>
     <row r="26">
@@ -2352,10 +2352,10 @@
         <v>1.6</v>
       </c>
       <c r="O26" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P26" t="n">
-        <v>104.4402940928782</v>
+        <v>97.85515876927929</v>
       </c>
       <c r="Q26" t="n">
         <v>-1.438970000000012</v>
@@ -2364,10 +2364,10 @@
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>79.90620722186421</v>
+        <v>76.28021440487922</v>
       </c>
       <c r="T26" t="n">
-        <v>79.90620722186421</v>
+        <v>76.28021440487922</v>
       </c>
     </row>
     <row r="27">
@@ -2426,10 +2426,10 @@
         <v>4.1</v>
       </c>
       <c r="O27" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P27" t="n">
-        <v>97.53621840096876</v>
+        <v>90.9496136210402</v>
       </c>
       <c r="Q27" t="n">
         <v>-1.438970000000012</v>
@@ -2438,10 +2438,10 @@
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>74.98951920332706</v>
+        <v>71.72616574473442</v>
       </c>
       <c r="T27" t="n">
-        <v>74.98951920332706</v>
+        <v>71.72616574473442</v>
       </c>
     </row>
     <row r="28">
@@ -2500,10 +2500,10 @@
         <v>4.199999999999999</v>
       </c>
       <c r="O28" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P28" t="n">
-        <v>97.26005537329239</v>
+        <v>90.67339181511063</v>
       </c>
       <c r="Q28" t="n">
         <v>1.867959999999982</v>
@@ -2512,10 +2512,10 @@
         <v>0</v>
       </c>
       <c r="S28" t="n">
-        <v>77.14785817942834</v>
+        <v>73.72484829538226</v>
       </c>
       <c r="T28" t="n">
-        <v>77.14785817942834</v>
+        <v>73.72484829538226</v>
       </c>
     </row>
     <row r="29">
@@ -2574,10 +2574,10 @@
         <v>5.949999999999999</v>
       </c>
       <c r="O29" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P29" t="n">
-        <v>92.42720238895575</v>
+        <v>85.83951021134328</v>
       </c>
       <c r="Q29" t="n">
         <v>-2.541280000000015</v>
@@ -2586,10 +2586,10 @@
         <v>0</v>
       </c>
       <c r="S29" t="n">
-        <v>70.56616790399532</v>
+        <v>67.62922157054273</v>
       </c>
       <c r="T29" t="n">
-        <v>70.56616790399532</v>
+        <v>67.62922157054273</v>
       </c>
     </row>
     <row r="30">
@@ -2648,10 +2648,10 @@
         <v>7.199999999999999</v>
       </c>
       <c r="O30" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P30" t="n">
-        <v>88.97516454300101</v>
+        <v>82.38673763722373</v>
       </c>
       <c r="Q30" t="n">
         <v>-1.438970000000012</v>
@@ -2660,10 +2660,10 @@
         <v>0</v>
       </c>
       <c r="S30" t="n">
-        <v>68.89282606034099</v>
+        <v>66.07914540615488</v>
       </c>
       <c r="T30" t="n">
-        <v>68.89282606034099</v>
+        <v>66.07914540615488</v>
       </c>
     </row>
     <row r="31">
@@ -2722,10 +2722,10 @@
         <v>9.199999999999999</v>
       </c>
       <c r="O31" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P31" t="n">
-        <v>83.45190398947342</v>
+        <v>76.86230151863246</v>
       </c>
       <c r="Q31" t="n">
         <v>1.867959999999982</v>
@@ -2734,10 +2734,10 @@
         <v>0</v>
       </c>
       <c r="S31" t="n">
-        <v>67.31448214235404</v>
+        <v>64.61675097509267</v>
       </c>
       <c r="T31" t="n">
-        <v>67.31448214235404</v>
+        <v>64.61675097509267</v>
       </c>
     </row>
     <row r="32">
@@ -2796,10 +2796,10 @@
         <v>13.7</v>
       </c>
       <c r="O32" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P32" t="n">
-        <v>71.02456774403635</v>
+        <v>64.43232025180211</v>
       </c>
       <c r="Q32" t="n">
         <v>-1.438970000000012</v>
@@ -2808,10 +2808,10 @@
         <v>0</v>
       </c>
       <c r="S32" t="n">
-        <v>56.10943721214443</v>
+        <v>54.23861888977843</v>
       </c>
       <c r="T32" t="n">
-        <v>56.10943721214443</v>
+        <v>54.23861888977843</v>
       </c>
     </row>
     <row r="33">
@@ -2872,10 +2872,10 @@
         <v>0</v>
       </c>
       <c r="O33" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P33" t="n">
-        <v>67.33771221119183</v>
+        <v>62.26700856676003</v>
       </c>
       <c r="Q33" t="n">
         <v>-0.3366600000000091</v>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="S33" t="n">
-        <v>54.26887163584412</v>
+        <v>53.53759365634961</v>
       </c>
       <c r="T33" t="n">
-        <v>54.26887163584412</v>
+        <v>53.53759365634961</v>
       </c>
     </row>
     <row r="34">
@@ -2946,10 +2946,10 @@
         <v>1.5</v>
       </c>
       <c r="O34" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P34" t="n">
-        <v>64.66054786882917</v>
+        <v>59.60058988347434</v>
       </c>
       <c r="Q34" t="n">
         <v>-2.541280000000015</v>
@@ -2958,10 +2958,10 @@
         <v>0</v>
       </c>
       <c r="S34" t="n">
-        <v>50.79234390696889</v>
+        <v>50.32525535243058</v>
       </c>
       <c r="T34" t="n">
-        <v>50.79234390696889</v>
+        <v>50.32525535243058</v>
       </c>
     </row>
     <row r="35">
@@ -3020,10 +3020,10 @@
         <v>2</v>
       </c>
       <c r="O35" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P35" t="n">
-        <v>63.76815975470828</v>
+        <v>58.71178365571245</v>
       </c>
       <c r="Q35" t="n">
         <v>-2.541280000000015</v>
@@ -3032,10 +3032,10 @@
         <v>0</v>
       </c>
       <c r="S35" t="n">
-        <v>50.15683610775331</v>
+        <v>49.73910802824727</v>
       </c>
       <c r="T35" t="n">
-        <v>50.15683610775331</v>
+        <v>49.73910802824727</v>
       </c>
     </row>
     <row r="36">
@@ -3094,10 +3094,10 @@
         <v>2.75</v>
       </c>
       <c r="O36" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P36" t="n">
-        <v>62.42957758352694</v>
+        <v>57.37857431406961</v>
       </c>
       <c r="Q36" t="n">
         <v>-2.541280000000015</v>
@@ -3106,10 +3106,10 @@
         <v>0</v>
       </c>
       <c r="S36" t="n">
-        <v>49.20357440892995</v>
+        <v>48.8598870419723</v>
       </c>
       <c r="T36" t="n">
-        <v>49.20357440892995</v>
+        <v>48.8598870419723</v>
       </c>
     </row>
     <row r="37">
@@ -3168,10 +3168,10 @@
         <v>2.85</v>
       </c>
       <c r="O37" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P37" t="n">
-        <v>62.25109996070277</v>
+        <v>57.20081306851723</v>
       </c>
       <c r="Q37" t="n">
         <v>-1.438970000000012</v>
@@ -3180,10 +3180,10 @@
         <v>0</v>
       </c>
       <c r="S37" t="n">
-        <v>49.8614750147011</v>
+        <v>49.46960574282018</v>
       </c>
       <c r="T37" t="n">
-        <v>49.8614750147011</v>
+        <v>49.46960574282018</v>
       </c>
     </row>
     <row r="38">
@@ -3242,10 +3242,10 @@
         <v>3.6</v>
       </c>
       <c r="O38" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P38" t="n">
-        <v>60.91251778952144</v>
+        <v>55.86760372687439</v>
       </c>
       <c r="Q38" t="n">
         <v>-0.3366600000000091</v>
@@ -3254,10 +3254,10 @@
         <v>0</v>
       </c>
       <c r="S38" t="n">
-        <v>49.693215481492</v>
+        <v>49.31733292222975</v>
       </c>
       <c r="T38" t="n">
-        <v>49.693215481492</v>
+        <v>49.31733292222975</v>
       </c>
     </row>
     <row r="39">
@@ -3316,10 +3316,10 @@
         <v>4.35</v>
       </c>
       <c r="O39" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P39" t="n">
-        <v>59.5739356183401</v>
+        <v>54.53439438523154</v>
       </c>
       <c r="Q39" t="n">
         <v>-2.541280000000015</v>
@@ -3328,10 +3328,10 @@
         <v>0</v>
       </c>
       <c r="S39" t="n">
-        <v>47.16994945144013</v>
+        <v>46.98421560458569</v>
       </c>
       <c r="T39" t="n">
-        <v>47.16994945144013</v>
+        <v>46.98421560458569</v>
       </c>
     </row>
     <row r="40">
@@ -3390,10 +3390,10 @@
         <v>4.85</v>
       </c>
       <c r="O40" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P40" t="n">
-        <v>58.68154750421922</v>
+        <v>53.64558815746965</v>
       </c>
       <c r="Q40" t="n">
         <v>-1.438970000000012</v>
@@ -3402,10 +3402,10 @@
         <v>0</v>
       </c>
       <c r="S40" t="n">
-        <v>47.31944381783881</v>
+        <v>47.12501644608693</v>
       </c>
       <c r="T40" t="n">
-        <v>47.31944381783881</v>
+        <v>47.12501644608693</v>
       </c>
     </row>
     <row r="41">
@@ -3464,10 +3464,10 @@
         <v>12.35</v>
       </c>
       <c r="O41" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P41" t="n">
-        <v>45.2957257924059</v>
+        <v>40.31349474104124</v>
       </c>
       <c r="Q41" t="n">
         <v>-2.541280000000015</v>
@@ -3476,10 +3476,10 @@
         <v>0</v>
       </c>
       <c r="S41" t="n">
-        <v>37.00182466399097</v>
+        <v>37.60585841765268</v>
       </c>
       <c r="T41" t="n">
-        <v>37.00182466399097</v>
+        <v>37.60585841765268</v>
       </c>
     </row>
     <row r="42">
@@ -3540,10 +3540,10 @@
         <v>0</v>
       </c>
       <c r="O42" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P42" t="n">
-        <v>137.8152797638106</v>
+        <v>135.8205578618974</v>
       </c>
       <c r="Q42" t="n">
         <v>-3.643590000000017</v>
@@ -3552,10 +3552,10 @@
         <v>0</v>
       </c>
       <c r="S42" t="n">
-        <v>102.1039597185939</v>
+        <v>99.86362811320892</v>
       </c>
       <c r="T42" t="n">
-        <v>102.1039597185939</v>
+        <v>99.86362811320892</v>
       </c>
     </row>
     <row r="43">
@@ -3614,10 +3614,10 @@
         <v>0.15</v>
       </c>
       <c r="O43" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P43" t="n">
-        <v>137.4766242806008</v>
+        <v>135.4827455184412</v>
       </c>
       <c r="Q43" t="n">
         <v>-2.541280000000015</v>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="S43" t="n">
-        <v>102.6477908091777</v>
+        <v>100.3677967854469</v>
       </c>
       <c r="T43" t="n">
-        <v>102.6477908091777</v>
+        <v>100.3677967854469</v>
       </c>
     </row>
     <row r="44">
@@ -3688,10 +3688,10 @@
         <v>0.25</v>
       </c>
       <c r="O44" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P44" t="n">
-        <v>137.250853958461</v>
+        <v>135.2575372894704</v>
       </c>
       <c r="Q44" t="n">
         <v>-2.541280000000015</v>
@@ -3700,10 +3700,10 @@
         <v>0</v>
       </c>
       <c r="S44" t="n">
-        <v>102.4870100924907</v>
+        <v>100.2192771231492</v>
       </c>
       <c r="T44" t="n">
-        <v>102.4870100924907</v>
+        <v>100.2192771231492</v>
       </c>
     </row>
     <row r="45">
@@ -3762,10 +3762,10 @@
         <v>2.25</v>
       </c>
       <c r="O45" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P45" t="n">
-        <v>132.7354475156642</v>
+        <v>130.7533727100542</v>
       </c>
       <c r="Q45" t="n">
         <v>-2.541280000000015</v>
@@ -3774,10 +3774,10 @@
         <v>0</v>
       </c>
       <c r="S45" t="n">
-        <v>99.27139575875155</v>
+        <v>97.2488838771949</v>
       </c>
       <c r="T45" t="n">
-        <v>99.27139575875155</v>
+        <v>97.2488838771949</v>
       </c>
     </row>
     <row r="46">
@@ -3836,10 +3836,10 @@
         <v>2.5</v>
       </c>
       <c r="O46" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P46" t="n">
-        <v>132.1710217103146</v>
+        <v>130.1903521376272</v>
       </c>
       <c r="Q46" t="n">
         <v>-2.541280000000015</v>
@@ -3848,10 +3848,10 @@
         <v>0</v>
       </c>
       <c r="S46" t="n">
-        <v>98.86944396703413</v>
+        <v>96.87758472145062</v>
       </c>
       <c r="T46" t="n">
-        <v>98.86944396703413</v>
+        <v>96.87758472145062</v>
       </c>
     </row>
     <row r="47">
@@ -3910,10 +3910,10 @@
         <v>3.5</v>
       </c>
       <c r="O47" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P47" t="n">
-        <v>129.9133184889162</v>
+        <v>127.9382698479192</v>
       </c>
       <c r="Q47" t="n">
         <v>4.072579999999988</v>
@@ -3922,10 +3922,10 @@
         <v>0</v>
       </c>
       <c r="S47" t="n">
-        <v>101.9716497938501</v>
+        <v>99.75407709258074</v>
       </c>
       <c r="T47" t="n">
-        <v>101.9716497938501</v>
+        <v>99.75407709258074</v>
       </c>
     </row>
     <row r="48">
@@ -3984,10 +3984,10 @@
         <v>4.25</v>
       </c>
       <c r="O48" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P48" t="n">
-        <v>128.2200410728674</v>
+        <v>126.2492081306381</v>
       </c>
       <c r="Q48" t="n">
         <v>-2.541280000000015</v>
@@ -3996,10 +3996,10 @@
         <v>0</v>
       </c>
       <c r="S48" t="n">
-        <v>96.05578142501236</v>
+        <v>94.27849063124064</v>
       </c>
       <c r="T48" t="n">
-        <v>96.05578142501236</v>
+        <v>94.27849063124064</v>
       </c>
     </row>
     <row r="49">
@@ -4058,10 +4058,10 @@
         <v>4.28</v>
       </c>
       <c r="O49" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P49" t="n">
-        <v>128.1523099762254</v>
+        <v>126.1816456619469</v>
       </c>
       <c r="Q49" t="n">
         <v>-3.643590000000017</v>
@@ -4070,10 +4070,10 @@
         <v>0</v>
       </c>
       <c r="S49" t="n">
-        <v>95.22254504439201</v>
+        <v>93.50698656686679</v>
       </c>
       <c r="T49" t="n">
-        <v>95.22254504439201</v>
+        <v>93.50698656686679</v>
       </c>
     </row>
     <row r="50">
@@ -4132,10 +4132,10 @@
         <v>5.78</v>
       </c>
       <c r="O50" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P50" t="n">
-        <v>124.7657551441278</v>
+        <v>122.8035222273848</v>
       </c>
       <c r="Q50" t="n">
         <v>-2.541280000000015</v>
@@ -4144,10 +4144,10 @@
         <v>0</v>
       </c>
       <c r="S50" t="n">
-        <v>93.59583645970186</v>
+        <v>92.00613979808564</v>
       </c>
       <c r="T50" t="n">
-        <v>93.59583645970186</v>
+        <v>92.00613979808564</v>
       </c>
     </row>
     <row r="51">
@@ -4206,10 +4206,10 @@
         <v>8.780000000000001</v>
       </c>
       <c r="O51" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P51" t="n">
-        <v>117.9926454799326</v>
+        <v>116.0472753582606</v>
       </c>
       <c r="Q51" t="n">
         <v>-0.3366600000000091</v>
@@ -4218,10 +4218,10 @@
         <v>0</v>
       </c>
       <c r="S51" t="n">
-        <v>90.34241929032157</v>
+        <v>89.00444626052332</v>
       </c>
       <c r="T51" t="n">
-        <v>90.34241929032157</v>
+        <v>89.00444626052332</v>
       </c>
     </row>
     <row r="52">
@@ -4280,10 +4280,10 @@
         <v>11.28</v>
       </c>
       <c r="O52" t="n">
-        <v>0.1749505941233769</v>
+        <v>0.2805563371141229</v>
       </c>
       <c r="P52" t="n">
-        <v>112.3483874264366</v>
+        <v>110.4170696339904</v>
       </c>
       <c r="Q52" t="n">
         <v>1.867959999999982</v>
@@ -4292,10 +4292,10 @@
         <v>0</v>
       </c>
       <c r="S52" t="n">
-        <v>87.89290570437609</v>
+        <v>86.74535103444957</v>
       </c>
       <c r="T52" t="n">
-        <v>87.89290570437609</v>
+        <v>86.74535103444957</v>
       </c>
     </row>
   </sheetData>

</xml_diff>